<commit_message>
enhance guest entry form with additional fields and improved styling
</commit_message>
<xml_diff>
--- a/hotelmode/data.xlsx
+++ b/hotelmode/data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,89 +407,26 @@
         <v>age</v>
       </c>
       <c r="C1" t="str">
+        <v>mak</v>
+      </c>
+      <c r="D1" t="str">
         <v>email</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Test</v>
+        <v>NNNNNNN</v>
       </c>
       <c r="B2" t="str">
-        <v>22</v>
-      </c>
-      <c r="C2" t="str">
-        <v>test@example.com</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>NNNNNNN</v>
-      </c>
-      <c r="B3" t="str">
         <v>5</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D2" t="str">
         <v>abenezerdaniel2wb0@gmail.com</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Abenezer Daniel</v>
-      </c>
-      <c r="B4" t="str">
-        <v>5</v>
-      </c>
-      <c r="C4" t="str">
-        <v>abenezerdaniel2wb0@gmail.com</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Alice</v>
-      </c>
-      <c r="B5" t="str">
-        <v>31</v>
-      </c>
-      <c r="C5" t="str">
-        <v>alice@example.com</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Bob</v>
-      </c>
-      <c r="B6" t="str">
-        <v>44</v>
-      </c>
-      <c r="C6" t="str">
-        <v>bob@example.com</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>ab</v>
-      </c>
-      <c r="B7" t="str">
-        <v>5</v>
-      </c>
-      <c r="C7" t="str">
-        <v>abenezerdaniel2wb0@gmail.com</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>nm</v>
-      </c>
-      <c r="B8" t="str">
-        <v>5</v>
-      </c>
-      <c r="C8" t="str">
-        <v>hhhhh</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update guest entry form with new fields, theme toggle, and data handling improvements
</commit_message>
<xml_diff>
--- a/hotelmode/data.xlsx
+++ b/hotelmode/data.xlsx
@@ -397,36 +397,147 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>name</v>
+        <v>fs</v>
       </c>
       <c r="B1" t="str">
-        <v>age</v>
+        <v>goods</v>
       </c>
       <c r="C1" t="str">
-        <v>mak</v>
+        <v>amount</v>
       </c>
       <c r="D1" t="str">
-        <v>email</v>
+        <v>price</v>
+      </c>
+      <c r="E1" t="str">
+        <v>sums</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>NNNNNNN</v>
+        <v>fs30004</v>
       </c>
       <c r="B2" t="str">
-        <v>5</v>
-      </c>
-      <c r="D2" t="str">
-        <v>abenezerdaniel2wb0@gmail.com</v>
+        <v>dulet</v>
+      </c>
+      <c r="C2" t="str">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>20</v>
+      </c>
+      <c r="E2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fs30004</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Areqe double</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>20</v>
+      </c>
+      <c r="E3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fs30008</v>
+      </c>
+      <c r="B4" t="str">
+        <v>tegabino</v>
+      </c>
+      <c r="C4" t="str">
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>fs30004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>beer</v>
+      </c>
+      <c r="C5" t="str">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>20</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>fs30004</v>
+      </c>
+      <c r="B6" t="str">
+        <v>beer</v>
+      </c>
+      <c r="C6" t="str">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>20</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>fs30004</v>
+      </c>
+      <c r="B7" t="str">
+        <v>beer</v>
+      </c>
+      <c r="C7" t="str">
+        <v>40</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>fs30004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>heinken</v>
+      </c>
+      <c r="C8" t="str">
+        <v>14</v>
+      </c>
+      <c r="D8">
+        <v>20</v>
+      </c>
+      <c r="E8">
+        <v>280</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>